<commit_message>
complete the last pie chart
</commit_message>
<xml_diff>
--- a/employees_data.xlsx
+++ b/employees_data.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="Employees" sheetId="1" r:id="rId1"/>
     <sheet name="Products" sheetId="2" r:id="rId2"/>
+    <sheet name="Buner Employees" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="266" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="159">
   <si>
     <t>ID</t>
   </si>
@@ -48,6 +49,12 @@
     <t>COntact</t>
   </si>
   <si>
+    <t>city</t>
+  </si>
+  <si>
+    <t>Count</t>
+  </si>
+  <si>
     <t>Ali</t>
   </si>
   <si>
@@ -120,6 +127,9 @@
     <t>03128462715</t>
   </si>
   <si>
+    <t>Buner</t>
+  </si>
+  <si>
     <t>Ayan</t>
   </si>
   <si>
@@ -385,9 +395,6 @@
   </si>
   <si>
     <t>850000</t>
-  </si>
-  <si>
-    <t>Buner</t>
   </si>
   <si>
     <t>KHAN KHAN</t>
@@ -1202,6 +1209,293 @@
 </styleSheet>
 </file>
 
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:date1904 val="0"/>
+  <c:lang val="zh-CN"/>
+  <c:roundedCorners val="0"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
+      <c14:style val="102"/>
+    </mc:Choice>
+    <mc:Fallback>
+      <c:style val="2"/>
+    </mc:Fallback>
+  </mc:AlternateContent>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="en-US" sz="1800" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="+mn-lt"/>
+                <a:ea typeface="+mn-ea"/>
+                <a:cs typeface="+mn-cs"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>Employees by city</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:pieChart>
+        <c:varyColors val="1"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Employees!$H$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Count</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln>
+              <a:noFill/>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </c:spPr>
+          <c:explosion val="0"/>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:ln>
+                <a:noFill/>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:delete val="1"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>Employees!$G$2:$G$8</c:f>
+              <c:strCache>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>BUNER</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Mardan</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Swat</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Charsadda</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Nowshera</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Peshawar</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Buner</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>Employees!$H$2:$H$8</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="7"/>
+                <c:pt idx="0">
+                  <c:v>1</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>11</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>9</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>10</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:dLbls>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="0"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:showLeaderLines val="1"/>
+        </c:dLbls>
+        <c:firstSliceAng val="0"/>
+      </c:pieChart>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="r"/>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="0" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr lang="en-US" sz="1000" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+    <c:extLst>
+      <c:ext uri="{0b15fc19-7d7d-44ad-8c2d-2c3a37ce22c3}">
+        <chartProps xmlns="https://web.wps.cn/et/2018/main" chartId="{b023240b-5d5d-435c-948b-4eaa7334c46f}"/>
+      </c:ext>
+    </c:extLst>
+  </c:chart>
+  <c:txPr>
+    <a:bodyPr/>
+    <a:lstStyle/>
+    <a:p>
+      <a:pPr>
+        <a:defRPr lang="en-US"/>
+      </a:pPr>
+    </a:p>
+  </c:txPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="5400000" cy="2611100"/>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="5657850" y="184150"/>
+        <a:ext cx="5399405" cy="2610485"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1487,10 +1781,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="5"/>
+  <dimension ref="A1:H54"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelCol="7"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1509,305 +1803,353 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D2">
         <v>50000</v>
       </c>
       <c r="E2" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>10</v>
+      </c>
+      <c r="H2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D3">
         <v>45000</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>15</v>
+      </c>
+      <c r="G3" t="s">
+        <v>14</v>
+      </c>
+      <c r="H3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D4">
         <v>55000</v>
       </c>
       <c r="E4" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F4" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>60000</v>
       </c>
       <c r="E5" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>22</v>
+      </c>
+      <c r="G5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H5">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D6">
         <v>47000</v>
       </c>
       <c r="E6" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>26</v>
+      </c>
+      <c r="G6" t="s">
+        <v>25</v>
+      </c>
+      <c r="H6">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>49000</v>
       </c>
       <c r="E7" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
+        <v>29</v>
+      </c>
+      <c r="G7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D8">
         <v>62000</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F8" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
+        <v>31</v>
+      </c>
+      <c r="G8" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D9">
         <v>53000</v>
       </c>
       <c r="E9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F9" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D10">
         <v>51000</v>
       </c>
       <c r="E10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F10" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D11">
         <v>65000</v>
       </c>
       <c r="E11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D12">
         <v>46000</v>
       </c>
       <c r="E12" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C13" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D13">
         <v>58000</v>
       </c>
       <c r="E13" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D14">
         <v>50000</v>
       </c>
       <c r="E14" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C15" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D15">
         <v>70000</v>
       </c>
       <c r="E15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F15" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="C16" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D16">
         <v>48000</v>
       </c>
       <c r="E16" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F16" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -1815,19 +2157,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C17" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D17">
         <v>56000</v>
       </c>
       <c r="E17" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F17" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -1835,19 +2177,19 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C18" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D18">
         <v>63000</v>
       </c>
       <c r="E18" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F18" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -1855,19 +2197,19 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="C19" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D19">
         <v>52000</v>
       </c>
       <c r="E19" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F19" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -1875,19 +2217,19 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C20" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D20">
         <v>47000</v>
       </c>
       <c r="E20" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F20" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -1895,19 +2237,19 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C21" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D21">
         <v>68000</v>
       </c>
       <c r="E21" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F21" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -1915,19 +2257,19 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C22" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D22">
         <v>59000</v>
       </c>
       <c r="E22" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F22" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -1935,19 +2277,19 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="C23" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D23">
         <v>54000</v>
       </c>
       <c r="E23" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F23" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -1955,19 +2297,19 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D24">
         <v>50000</v>
       </c>
       <c r="E24" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F24" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -1975,19 +2317,19 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C25" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D25">
         <v>72000</v>
       </c>
       <c r="E25" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F25" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -1995,19 +2337,19 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C26" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D26">
         <v>61000</v>
       </c>
       <c r="E26" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F26" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2015,19 +2357,19 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D27">
         <v>53000</v>
       </c>
       <c r="E27" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F27" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2035,19 +2377,19 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C28" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D28">
         <v>49000</v>
       </c>
       <c r="E28" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F28" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -2055,19 +2397,19 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C29" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D29">
         <v>66000</v>
       </c>
       <c r="E29" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F29" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -2075,19 +2417,19 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C30" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D30">
         <v>57000</v>
       </c>
       <c r="E30" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F30" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -2095,19 +2437,19 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C31" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D31">
         <v>55000</v>
       </c>
       <c r="E31" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F31" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -2115,19 +2457,19 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D32">
         <v>51000</v>
       </c>
       <c r="E32" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F32" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -2135,19 +2477,19 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C33" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D33">
         <v>74000</v>
       </c>
       <c r="E33" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F33" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -2155,19 +2497,19 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C34" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D34">
         <v>62000</v>
       </c>
       <c r="E34" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F34" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -2175,19 +2517,19 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C35" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D35">
         <v>56000</v>
       </c>
       <c r="E35" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F35" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -2195,19 +2537,19 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C36" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D36">
         <v>52000</v>
       </c>
       <c r="E36" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F36" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2215,19 +2557,19 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C37" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D37">
         <v>69000</v>
       </c>
       <c r="E37" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F37" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -2235,19 +2577,19 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C38" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D38">
         <v>60000</v>
       </c>
       <c r="E38" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F38" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -2255,19 +2597,19 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C39" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D39">
         <v>54000</v>
       </c>
       <c r="E39" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F39" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -2275,19 +2617,19 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C40" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D40">
         <v>50000</v>
       </c>
       <c r="E40" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F40" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -2295,19 +2637,19 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C41" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D41">
         <v>76000</v>
       </c>
       <c r="E41" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F41" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -2315,19 +2657,19 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C42" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D42">
         <v>63000</v>
       </c>
       <c r="E42" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F42" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -2335,19 +2677,19 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C43" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D43">
         <v>57000</v>
       </c>
       <c r="E43" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F43" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -2355,19 +2697,19 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C44" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D44">
         <v>53000</v>
       </c>
       <c r="E44" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F44" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -2375,19 +2717,19 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C45" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D45">
         <v>71000</v>
       </c>
       <c r="E45" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F45" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -2395,19 +2737,19 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C46" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D46">
         <v>64000</v>
       </c>
       <c r="E46" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F46" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -2415,19 +2757,19 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="C47" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D47">
         <v>58000</v>
       </c>
       <c r="E47" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="F47" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -2435,19 +2777,19 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="C48" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D48">
         <v>52000</v>
       </c>
       <c r="E48" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F48" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -2455,19 +2797,19 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="C49" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="D49">
         <v>73000</v>
       </c>
       <c r="E49" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F49" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -2475,19 +2817,19 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C50" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="D50">
         <v>65000</v>
       </c>
       <c r="E50" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F50" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -2495,19 +2837,19 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="C51" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D51">
         <v>59000</v>
       </c>
       <c r="E51" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F51" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -2515,21 +2857,21 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="C52" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D52" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="E52" t="s">
-        <v>119</v>
+        <v>32</v>
       </c>
     </row>
     <row r="53" ht="19" spans="1:6">
       <c r="A53" s="2" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D53">
         <f>SUM(D2:D52)</f>
@@ -2538,12 +2880,13 @@
     </row>
     <row r="54" spans="1:6">
       <c r="A54" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -2555,48 +2898,48 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D1" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="E1" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" t="s">
+        <v>131</v>
+      </c>
+      <c r="C2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2" t="s">
+        <v>132</v>
+      </c>
+      <c r="F2" t="s">
         <v>128</v>
       </c>
-      <c r="B2" t="s">
+      <c r="G2" t="s">
         <v>129</v>
-      </c>
-      <c r="C2" t="s">
-        <v>123</v>
-      </c>
-      <c r="D2" t="s">
-        <v>124</v>
-      </c>
-      <c r="E2" t="s">
-        <v>130</v>
-      </c>
-      <c r="F2" t="s">
-        <v>126</v>
-      </c>
-      <c r="G2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -2604,10 +2947,10 @@
         <v>1</v>
       </c>
       <c r="B3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D3">
         <v>85000</v>
@@ -2627,10 +2970,10 @@
         <v>2</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D4">
         <v>1200</v>
@@ -2650,10 +2993,10 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C5" t="s">
         <v>134</v>
-      </c>
-      <c r="C5" t="s">
-        <v>132</v>
       </c>
       <c r="D5">
         <v>2500</v>
@@ -2673,10 +3016,10 @@
         <v>4</v>
       </c>
       <c r="B6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D6">
         <v>3500</v>
@@ -2696,10 +3039,10 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C7" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D7">
         <v>28000</v>
@@ -2719,10 +3062,10 @@
         <v>6</v>
       </c>
       <c r="B8" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D8">
         <v>22000</v>
@@ -2742,10 +3085,10 @@
         <v>7</v>
       </c>
       <c r="B9" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D9">
         <v>1500</v>
@@ -2765,10 +3108,10 @@
         <v>8</v>
       </c>
       <c r="B10" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C10" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D10">
         <v>3000</v>
@@ -2788,10 +3131,10 @@
         <v>9</v>
       </c>
       <c r="B11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="D11">
         <v>12000</v>
@@ -2811,10 +3154,10 @@
         <v>10</v>
       </c>
       <c r="B12" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="C12" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D12">
         <v>45000</v>
@@ -2834,10 +3177,10 @@
         <v>11</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D13">
         <v>5500</v>
@@ -2857,10 +3200,10 @@
         <v>12</v>
       </c>
       <c r="B14" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C14" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D14">
         <v>6500</v>
@@ -2880,10 +3223,10 @@
         <v>13</v>
       </c>
       <c r="B15" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C15" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D15">
         <v>4000</v>
@@ -2903,10 +3246,10 @@
         <v>14</v>
       </c>
       <c r="B16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C16" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D16">
         <v>7000</v>
@@ -2926,10 +3269,10 @@
         <v>15</v>
       </c>
       <c r="B17" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C17" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D17">
         <v>9500</v>
@@ -2949,10 +3292,10 @@
         <v>16</v>
       </c>
       <c r="B18" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C18" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D18">
         <v>7500</v>
@@ -2972,10 +3315,10 @@
         <v>17</v>
       </c>
       <c r="B19" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C19" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D19">
         <v>95000</v>
@@ -2995,10 +3338,10 @@
         <v>18</v>
       </c>
       <c r="B20" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C20" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D20">
         <v>14000</v>
@@ -3018,10 +3361,10 @@
         <v>19</v>
       </c>
       <c r="B21" t="s">
+        <v>157</v>
+      </c>
+      <c r="C21" t="s">
         <v>155</v>
-      </c>
-      <c r="C21" t="s">
-        <v>153</v>
       </c>
       <c r="D21">
         <v>55000</v>
@@ -3041,10 +3384,10 @@
         <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C22" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D22">
         <v>25000</v>
@@ -3057,6 +3400,43 @@
       </c>
       <c r="G22">
         <v>4.6</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A2:E6"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="5" outlineLevelCol="4"/>
+  <sheetData>
+    <row r="2" spans="1:5">
+      <c r="A2">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="B3" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="C4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="D5" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="E6" t="s">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>